<commit_message>
Added Fee waiver Supreme court to easy form spreadsheet
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEA27B28-853D-4604-BB22-676AD91A3581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDA89CC5-6C74-4220-8C16-7FD5E8C854D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
   <si>
     <t>name</t>
   </si>
@@ -397,6 +397,12 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/vacate-default-judgment-foreclosure</t>
+  </si>
+  <si>
+    <t>Fee waiver - Supreme Court of Illinois</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/fee-waiver-supreme-court-illinois</t>
   </si>
 </sst>
 </file>
@@ -759,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.77734375" customWidth="1"/>
@@ -944,321 +950,329 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>124</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>73</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>109</v>
+        <v>72</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>110</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>11</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>104</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>119</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>43</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>112</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>16</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>116</v>
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>123</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>81</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>106</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B63" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1270,46 +1284,46 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B21" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B52" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B25" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B56" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B45" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B53" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B26" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B57" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B46" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B48" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B26" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B29" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B57" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B39" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B40" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B38" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B37" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B33" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
-    <hyperlink ref="B31" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
+    <hyperlink ref="B49" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B27" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B30" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B58" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B40" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B41" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B39" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B38" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B34" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B32" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B53" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B42" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B50" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B54" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B51" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B54" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B43" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B51" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B55" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B52" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
-    <hyperlink ref="B23" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B46" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B61" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
-    <hyperlink ref="B30" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
+    <hyperlink ref="B24" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
+    <hyperlink ref="B47" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B62" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B31" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B59" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B47" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B27" r:id="rId36" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
-    <hyperlink ref="B24" r:id="rId37" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B62" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B43" r:id="rId39" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B60" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B48" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B28" r:id="rId36" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B25" r:id="rId37" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
+    <hyperlink ref="B63" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B44" r:id="rId39" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
     <hyperlink ref="B22" r:id="rId40" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
-    <hyperlink ref="B58" r:id="rId41" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
-    <hyperlink ref="B44" r:id="rId42" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
-    <hyperlink ref="B36" r:id="rId43" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
+    <hyperlink ref="B59" r:id="rId41" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B45" r:id="rId42" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
+    <hyperlink ref="B37" r:id="rId43" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Notice of Appeal to xlsx
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F52443C9-34A3-4C7E-8BA0-EAB3062240ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{937416F3-F766-4E7D-A770-59B0B756EB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="130">
   <si>
     <t>name</t>
   </si>
@@ -412,6 +409,12 @@
   </si>
   <si>
     <t>name_es</t>
+  </si>
+  <si>
+    <t>Notice of appeal</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/notice-appeal</t>
   </si>
 </sst>
 </file>
@@ -774,15 +777,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C63"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C64"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="49.81640625" customWidth="1"/>
-    <col min="2" max="2" width="104.453125" customWidth="1"/>
-    <col min="3" max="3" width="33.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.77734375" customWidth="1"/>
+    <col min="2" max="2" width="104.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -793,7 +796,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -801,7 +804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -809,7 +812,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -817,7 +820,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -825,7 +828,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>92</v>
       </c>
@@ -833,7 +836,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>107</v>
       </c>
@@ -841,7 +844,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>70</v>
       </c>
@@ -849,7 +852,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>90</v>
       </c>
@@ -857,7 +860,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>88</v>
       </c>
@@ -865,7 +868,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>84</v>
       </c>
@@ -873,7 +876,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -881,7 +884,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -889,7 +892,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -897,7 +900,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>102</v>
       </c>
@@ -905,7 +908,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -913,7 +916,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -921,7 +924,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -929,7 +932,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>122</v>
       </c>
@@ -937,7 +940,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -945,7 +948,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -953,7 +956,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>113</v>
       </c>
@@ -961,7 +964,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>124</v>
       </c>
@@ -969,7 +972,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -977,7 +980,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>109</v>
       </c>
@@ -985,7 +988,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -993,7 +996,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1001,7 +1004,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -1009,7 +1012,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>25</v>
       </c>
@@ -1017,7 +1020,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -1025,7 +1028,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>83</v>
       </c>
@@ -1033,7 +1036,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -1041,7 +1044,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>56</v>
       </c>
@@ -1049,246 +1052,254 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>44</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>119</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B38" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>46</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>63</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>111</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
         <v>117</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B46" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>100</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B47" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
         <v>80</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B48" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>98</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
         <v>27</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B50" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>74</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B51" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
         <v>62</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B52" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>68</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B53" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>9</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B54" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>61</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B55" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>64</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>76</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B57" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
         <v>14</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>34</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B59" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>115</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>96</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B61" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
         <v>101</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B62" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>78</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B63" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
         <v>106</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B64" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1300,46 +1311,47 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B21" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B53" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B54" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="B26" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B57" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B46" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B58" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B47" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B49" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B50" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
     <hyperlink ref="B27" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="B30" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B58" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B40" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B41" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B39" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B38" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B34" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B59" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B41" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B42" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B40" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B39" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B35" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
     <hyperlink ref="B32" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B54" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B43" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B51" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B55" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B52" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B55" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B44" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B52" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B56" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B53" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
     <hyperlink ref="B24" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B47" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B62" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B48" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B63" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
     <hyperlink ref="B31" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B60" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B48" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B61" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B49" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
     <hyperlink ref="B28" r:id="rId36" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
     <hyperlink ref="B25" r:id="rId37" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B63" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B44" r:id="rId39" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B64" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B45" r:id="rId39" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
     <hyperlink ref="B22" r:id="rId40" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
-    <hyperlink ref="B59" r:id="rId41" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
-    <hyperlink ref="B45" r:id="rId42" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
-    <hyperlink ref="B37" r:id="rId43" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
+    <hyperlink ref="B60" r:id="rId41" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B46" r:id="rId42" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
+    <hyperlink ref="B38" r:id="rId43" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
+    <hyperlink ref="B34" r:id="rId44" xr:uid="{B29F375F-3BA3-4878-A2B0-123B3CE62790}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>